<commit_message>
Actualización automática de resultados testigos
</commit_message>
<xml_diff>
--- a/testigos/GLOBAL/16._BOGOTA_D.C/001._BOGOTA_D.C/13._TEUSAQUILLO/df_testigos_total_13._TEUSAQUILLO.xlsx
+++ b/testigos/GLOBAL/16._BOGOTA_D.C/001._BOGOTA_D.C/13._TEUSAQUILLO/df_testigos_total_13._TEUSAQUILLO.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,7 +505,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="2" t="n">
+        <v>46057.54694444445</v>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>C.C.</t>
@@ -509,60 +515,128 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>123789456</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>JUAN</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JOSE</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>JIMENEZ</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>JULIO</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Juan.jose@gmail.com</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>573123789456</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>16. BOGOTA D.C.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>001. BOGOTA D.C.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>13. TEUSAQUILLO</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>02. SAN LUIS</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Votante y Testigo de mesa</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>C.C.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>159357426</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>ANTONIO</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>ARTURO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>ANTARES</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>ANGULO</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>g@g.com</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>573123456789</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>16. BOGOTA D.C.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>001. BOGOTA D.C.</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>13. TEUSAQUILLO</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>10. COLEGIO AMERICANO</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Votante y Testigo de mesa</t>
         </is>

</xml_diff>